<commit_message>
finished space heating, cooling, water heating
</commit_message>
<xml_diff>
--- a/[deprecated]/Residential/Ontario/Residential space cooling.xlsx
+++ b/[deprecated]/Residential/Ontario/Residential space cooling.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/daniel_posen_utoronto_ca/Documents/Academia/File Sharing/Alliance Mission - TEMOA/Full team - TEMOA/TEMOA model and data/Data sources/Buildings/Residential/Ontario/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/buildings_sector/[deprecated]/Residential/Ontario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:40009_{D5B80FD9-2AB7-47F2-AE61-4E4335F9F641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{384FBCFE-AAAA-4C33-A6D8-09047EE7F5A0}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:40009_{D5B80FD9-2AB7-47F2-AE61-4E4335F9F641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2736DAE7-839C-4329-8716-CBBA1598143D}"/>
   <bookViews>
-    <workbookView xWindow="15765" yWindow="3195" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand and Existing Capacity" sheetId="3" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="50">
   <si>
     <t>Residential Sector</t>
   </si>
@@ -320,19 +320,7 @@
     <t>2) Space cooling consumes only electricity.</t>
   </si>
   <si>
-    <t>Primary energy (PJ p.a.)</t>
-  </si>
-  <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Pop. Index</t>
-  </si>
-  <si>
-    <t>SPC demand (PJ p.a.)</t>
   </si>
   <si>
     <t>Technology</t>
@@ -344,16 +332,10 @@
     <t>R_SPC_CEN_EXS</t>
   </si>
   <si>
-    <t>Stock (x1000)</t>
-  </si>
-  <si>
     <t>Population index</t>
   </si>
   <si>
     <t>Unit cap.</t>
-  </si>
-  <si>
-    <t>(GW)</t>
   </si>
   <si>
     <t>(kBtu/h)</t>
@@ -366,15 +348,6 @@
   </si>
   <si>
     <t>PJ =</t>
-  </si>
-  <si>
-    <t>x GW</t>
-  </si>
-  <si>
-    <t>Annual CF</t>
-  </si>
-  <si>
-    <t>Exs cap. (GW)</t>
   </si>
   <si>
     <t>(Y)</t>
@@ -395,22 +368,38 @@
     <t>x Wh</t>
   </si>
   <si>
-    <t>2023 max annual PJ</t>
+    <t>c2a (PJ.Munit)</t>
+  </si>
+  <si>
+    <t>x GWy</t>
+  </si>
+  <si>
+    <t>Stock (Munit)</t>
+  </si>
+  <si>
+    <t>arb. C2a</t>
+  </si>
+  <si>
+    <t>acf</t>
+  </si>
+  <si>
+    <t>max act</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="#\ ##0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
     <numFmt numFmtId="167" formatCode="#,##0.000"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
-    <numFmt numFmtId="171" formatCode="0.000%"/>
+    <numFmt numFmtId="169" formatCode="0.000%"/>
+    <numFmt numFmtId="172" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -531,21 +520,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -580,9 +554,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -637,12 +611,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -681,10 +650,11 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="172" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -900,7 +870,7 @@
       <xdr:spPr bwMode="auto">
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="5048250" cy="571500"/>
+          <a:ext cx="7731919" cy="1202531"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1306,299 +1276,153 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A2:K10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" customWidth="1"/>
     <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" style="31"/>
+    <col min="9" max="9" width="9.140625" style="28"/>
     <col min="10" max="10" width="22.28515625" customWidth="1"/>
     <col min="11" max="11" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="14">
-        <v>2018</v>
-      </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-    </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2">
-        <f>'secondary energy'!U15*efficiency!U27*0.293071</f>
-        <v>4.3615729801956222</v>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3">
-        <f>'secondary energy'!U16*efficiency!U28*0.293071</f>
-        <v>86.32862363633761</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
+      <c r="A3" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="B5">
-        <f>SUM(B2:B3)</f>
-        <v>90.690196616533228</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
+      <c r="B3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="26">
+        <v>2020</v>
+      </c>
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3" s="26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="28">
-        <v>2018</v>
-      </c>
-      <c r="C7">
-        <v>2023</v>
-      </c>
-      <c r="D7" s="27">
-        <v>2025</v>
-      </c>
-      <c r="E7" s="27">
-        <v>2030</v>
-      </c>
-      <c r="F7" s="27">
-        <v>2035</v>
-      </c>
-      <c r="G7" s="27">
-        <v>2040</v>
-      </c>
-      <c r="H7" s="27">
-        <v>2045</v>
-      </c>
-      <c r="I7" s="27">
-        <v>2050</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="B8" s="29">
-        <v>1</v>
-      </c>
-      <c r="C8">
-        <v>1.0743186469040473</v>
-      </c>
-      <c r="D8">
-        <v>1.1068652861962205</v>
-      </c>
-      <c r="E8">
-        <v>1.1799676797964203</v>
-      </c>
-      <c r="F8">
-        <v>1.2445018578560998</v>
-      </c>
-      <c r="G8">
-        <v>1.3009849883605753</v>
-      </c>
-      <c r="H8">
-        <v>1.3513459681199482</v>
-      </c>
-      <c r="I8">
-        <v>1.3975416489705528</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="29">
-        <v>90.690196616533228</v>
-      </c>
-      <c r="C9" s="31">
-        <f>$B$9*C8/$B$8</f>
-        <v>97.430169316535995</v>
-      </c>
-      <c r="D9">
-        <f>$B$9*D8/$B$8</f>
-        <v>100.38183043315055</v>
-      </c>
-      <c r="E9">
-        <f t="shared" ref="E9:I9" si="0">$B$9*E8/$B$8</f>
-        <v>107.01150088189188</v>
-      </c>
-      <c r="F9">
-        <f t="shared" si="0"/>
-        <v>112.86411817861058</v>
-      </c>
-      <c r="G9">
-        <f t="shared" si="0"/>
-        <v>117.98658438957877</v>
-      </c>
-      <c r="H9">
-        <f t="shared" si="0"/>
-        <v>122.55383154575755</v>
-      </c>
-      <c r="I9">
-        <f t="shared" si="0"/>
-        <v>126.7433269249335</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>48</v>
-      </c>
-      <c r="C11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12">
-        <v>2020</v>
-      </c>
-      <c r="D12" s="27">
-        <v>2023</v>
-      </c>
-      <c r="E12" t="s">
-        <v>40</v>
-      </c>
-      <c r="F12" t="s">
-        <v>39</v>
-      </c>
-      <c r="G12" t="s">
-        <v>46</v>
-      </c>
-      <c r="J12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="30" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13">
+      <c r="B4">
         <v>9</v>
       </c>
-      <c r="C13">
-        <f>stock!W15</f>
-        <v>479.07</v>
-      </c>
-      <c r="D13">
-        <f>$D$16/$C$16*C13</f>
-        <v>500.08834341005331</v>
-      </c>
-      <c r="E13" s="51">
+      <c r="C4" s="26">
+        <f>stock!W15/1000</f>
+        <v>0.47907</v>
+      </c>
+      <c r="D4" s="48">
         <f>stock!W31/1000</f>
         <v>9.1720000000000006</v>
       </c>
-      <c r="F13" s="52">
-        <f>$B$18*E13</f>
-        <v>2.6880472120000005E-6</v>
-      </c>
-      <c r="G13" s="53">
-        <f>F13*D13*1000</f>
-        <v>1.3442610772570927</v>
-      </c>
-      <c r="J13">
-        <f>G13*$B$19</f>
-        <v>42.392617332379679</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14">
+      <c r="E4" s="52">
+        <f>$B$10*$B$9*D4*C4*1000000</f>
+        <v>40.610886962367175</v>
+      </c>
+      <c r="F4" s="26">
+        <v>1000</v>
+      </c>
+      <c r="G4" s="49">
+        <f>F4*C4</f>
+        <v>479.07</v>
+      </c>
+      <c r="H4" s="53">
+        <f>'secondary energy'!W15/'Demand and Existing Capacity'!G4</f>
+        <v>2.273212682906465E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5">
         <v>18</v>
       </c>
-      <c r="C14" s="31">
-        <f>stock!W16</f>
-        <v>4028.4560000000001</v>
-      </c>
-      <c r="D14" s="31">
-        <f>$D$16/$C$16*C14</f>
-        <v>4205.1973355465589</v>
-      </c>
-      <c r="E14" s="51">
+      <c r="C5" s="26">
+        <f>stock!W16/1000</f>
+        <v>4.0284560000000003</v>
+      </c>
+      <c r="D5" s="48">
         <f>stock!W32/1000</f>
         <v>33.198999999999998</v>
       </c>
-      <c r="F14" s="52">
-        <f>$B$18*E14</f>
-        <v>9.7296641290000017E-6</v>
-      </c>
-      <c r="G14" s="53">
-        <f>F14*D14*1000</f>
-        <v>40.915157671033739</v>
-      </c>
-      <c r="J14" s="31">
-        <f>G14*$B$19</f>
-        <v>1290.30041231372</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="K15" s="34" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" s="31">
-        <v>1</v>
-      </c>
-      <c r="D16" s="50">
-        <v>1.0438732198009755</v>
-      </c>
-      <c r="F16" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="G16" s="53">
-        <f>SUM(G13:G14)</f>
-        <v>42.259418748290834</v>
-      </c>
-      <c r="J16">
-        <f>SUM(J13:J14)</f>
-        <v>1332.6930296460996</v>
-      </c>
-      <c r="K16" s="55">
-        <f>C9/J16</f>
-        <v>7.3107735351785288E-2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="31">
+      <c r="E5" s="52">
+        <f>$B$10*$B$9*D5*C5*1000000</f>
+        <v>1236.0700397695116</v>
+      </c>
+      <c r="F5" s="26">
+        <v>1000</v>
+      </c>
+      <c r="G5" s="49">
+        <f>F5*C5</f>
+        <v>4028.4560000000001</v>
+      </c>
+      <c r="H5" s="53">
+        <f>'secondary energy'!W16/'Demand and Existing Capacity'!G5</f>
+        <v>5.980351529221121E-3</v>
+      </c>
+      <c r="J5" s="28"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K6" s="31"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="28"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="49"/>
+      <c r="K7" s="51"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="28">
         <f>0.293071*1000/1000000000</f>
         <v>2.9307100000000004E-7</v>
       </c>
-      <c r="C18" s="31" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="31">
+      <c r="C9" s="28" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="28">
         <f>8760*3600/1000000</f>
         <v>31.536000000000001</v>
       </c>
-      <c r="C19" s="31" t="s">
-        <v>44</v>
+      <c r="C10" s="28" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1682,7 +1506,7 @@
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A2" s="54" t="str" cm="1">
+      <c r="A2" s="50" t="str" cm="1">
         <f t="array" ref="A2:V3">efficiency!B23:W24</f>
         <v>Room (EER)1</v>
       </c>
@@ -1820,191 +1644,191 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <f>B2/$B$8</f>
         <v>2.7402158176393701</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="28">
         <f t="shared" ref="C5:V6" si="0">C2/$B$8</f>
         <v>2.7402158176393701</v>
       </c>
-      <c r="D5" s="31">
+      <c r="D5" s="28">
         <f t="shared" si="0"/>
         <v>2.7402158176393701</v>
       </c>
-      <c r="E5" s="31">
+      <c r="E5" s="28">
         <f t="shared" si="0"/>
         <v>2.7402158176393701</v>
       </c>
-      <c r="F5" s="31">
+      <c r="F5" s="28">
         <f t="shared" si="0"/>
         <v>2.7402158176393701</v>
       </c>
-      <c r="G5" s="31">
+      <c r="G5" s="28">
         <f t="shared" si="0"/>
         <v>2.7402158176393701</v>
       </c>
-      <c r="H5" s="31">
+      <c r="H5" s="28">
         <f t="shared" si="0"/>
         <v>3.1944761938255759</v>
       </c>
-      <c r="I5" s="31">
+      <c r="I5" s="28">
         <f t="shared" si="0"/>
         <v>3.1944761938255759</v>
       </c>
-      <c r="J5" s="31">
+      <c r="J5" s="28">
         <f t="shared" si="0"/>
         <v>3.1944761938255759</v>
       </c>
-      <c r="K5" s="31">
+      <c r="K5" s="28">
         <f t="shared" si="0"/>
         <v>3.1944761938255759</v>
       </c>
-      <c r="L5" s="31">
+      <c r="L5" s="28">
         <f t="shared" si="0"/>
         <v>3.5168545253125605</v>
       </c>
-      <c r="M5" s="31">
+      <c r="M5" s="28">
         <f t="shared" si="0"/>
         <v>3.5168545253125605</v>
       </c>
-      <c r="N5" s="31">
+      <c r="N5" s="28">
         <f t="shared" si="0"/>
         <v>3.5168545253125605</v>
       </c>
-      <c r="O5" s="31">
+      <c r="O5" s="28">
         <f t="shared" si="0"/>
         <v>3.5168545253125605</v>
       </c>
-      <c r="P5" s="31">
+      <c r="P5" s="28">
         <f t="shared" si="0"/>
         <v>3.5168545253125605</v>
       </c>
-      <c r="Q5" s="31">
+      <c r="Q5" s="28">
         <f t="shared" si="0"/>
         <v>3.5168545253125605</v>
       </c>
-      <c r="R5" s="31">
+      <c r="R5" s="28">
         <f t="shared" si="0"/>
         <v>3.5168545253125605</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="28">
         <f t="shared" si="0"/>
         <v>3.5168545253125605</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="28">
         <f t="shared" si="0"/>
         <v>3.5168545253125605</v>
       </c>
-      <c r="U5" s="31">
+      <c r="U5" s="28">
         <f t="shared" si="0"/>
         <v>3.5168545253125605</v>
       </c>
-      <c r="V5" s="31">
+      <c r="V5" s="28">
         <f t="shared" si="0"/>
         <v>3.5168545253125605</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="31">
+        <v>41</v>
+      </c>
+      <c r="B6" s="28">
         <f>B3/$B$8</f>
         <v>3.018633467559948</v>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="28">
         <f t="shared" si="0"/>
         <v>3.018633467559948</v>
       </c>
-      <c r="D6" s="31">
+      <c r="D6" s="28">
         <f t="shared" si="0"/>
         <v>3.018633467559948</v>
       </c>
-      <c r="E6" s="31">
+      <c r="E6" s="28">
         <f t="shared" si="0"/>
         <v>3.018633467559948</v>
       </c>
-      <c r="F6" s="31">
+      <c r="F6" s="28">
         <f t="shared" si="0"/>
         <v>3.018633467559948</v>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="28">
         <f t="shared" si="0"/>
         <v>3.018633467559948</v>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="J6" s="31">
+      <c r="J6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="K6" s="31">
+      <c r="K6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="L6" s="31">
+      <c r="L6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="M6" s="31">
+      <c r="M6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="N6" s="31">
+      <c r="N6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="O6" s="31">
+      <c r="O6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="P6" s="31">
+      <c r="P6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="Q6" s="31">
+      <c r="Q6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="R6" s="31">
+      <c r="R6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="T6" s="31">
+      <c r="T6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="U6" s="31">
+      <c r="U6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
-      <c r="V6" s="31">
+      <c r="V6" s="28">
         <f t="shared" si="0"/>
         <v>3.8099257357552738</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A8" s="34" t="s">
-        <v>51</v>
+      <c r="A8" s="31" t="s">
+        <v>42</v>
       </c>
       <c r="B8">
         <v>3.41214</v>
       </c>
       <c r="C8" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -3173,7 +2997,6 @@
     <row r="56" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="57" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -4215,1556 +4038,1556 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A1" s="31"/>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
-      <c r="N1" s="31"/>
-      <c r="O1" s="31"/>
-      <c r="P1" s="31"/>
-      <c r="Q1" s="31"/>
-      <c r="R1" s="31"/>
-      <c r="S1" s="31"/>
-      <c r="T1" s="31"/>
-      <c r="U1" s="31"/>
-      <c r="V1" s="31"/>
-      <c r="W1" s="31"/>
+      <c r="A1" s="28"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="28"/>
+      <c r="S1" s="28"/>
+      <c r="T1" s="28"/>
+      <c r="U1" s="28"/>
+      <c r="V1" s="28"/>
+      <c r="W1" s="28"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A2" s="31"/>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
-      <c r="R2" s="31"/>
-      <c r="S2" s="31"/>
-      <c r="T2" s="31"/>
-      <c r="U2" s="31"/>
-      <c r="V2" s="31"/>
-      <c r="W2" s="31"/>
+      <c r="A2" s="28"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+      <c r="P2" s="28"/>
+      <c r="Q2" s="28"/>
+      <c r="R2" s="28"/>
+      <c r="S2" s="28"/>
+      <c r="T2" s="28"/>
+      <c r="U2" s="28"/>
+      <c r="V2" s="28"/>
+      <c r="W2" s="28"/>
     </row>
     <row r="5" spans="1:23" ht="18" x14ac:dyDescent="0.25">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="34"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="34"/>
-      <c r="N5" s="34"/>
-      <c r="O5" s="34"/>
-      <c r="P5" s="31"/>
-      <c r="Q5" s="31"/>
-      <c r="R5" s="31"/>
-      <c r="S5" s="31"/>
-      <c r="T5" s="31"/>
-      <c r="U5" s="31"/>
-      <c r="V5" s="31"/>
-      <c r="W5" s="31"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
+      <c r="P5" s="28"/>
+      <c r="Q5" s="28"/>
+      <c r="R5" s="28"/>
+      <c r="S5" s="28"/>
+      <c r="T5" s="28"/>
+      <c r="U5" s="28"/>
+      <c r="V5" s="28"/>
+      <c r="W5" s="28"/>
     </row>
     <row r="6" spans="1:23" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="33"/>
-      <c r="B6" s="31"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
-      <c r="M6" s="34"/>
-      <c r="N6" s="34"/>
-      <c r="O6" s="34"/>
-      <c r="P6" s="31"/>
-      <c r="Q6" s="31"/>
-      <c r="R6" s="31"/>
-      <c r="S6" s="31"/>
-      <c r="T6" s="31"/>
-      <c r="U6" s="31"/>
-      <c r="V6" s="31"/>
-      <c r="W6" s="31"/>
+      <c r="A6" s="30"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="31"/>
+      <c r="L6" s="31"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="31"/>
+      <c r="O6" s="31"/>
+      <c r="P6" s="28"/>
+      <c r="Q6" s="28"/>
+      <c r="R6" s="28"/>
+      <c r="S6" s="28"/>
+      <c r="T6" s="28"/>
+      <c r="U6" s="28"/>
+      <c r="V6" s="28"/>
+      <c r="W6" s="28"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="31"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="31"/>
-      <c r="G7" s="31"/>
-      <c r="H7" s="31"/>
-      <c r="I7" s="31"/>
-      <c r="J7" s="31"/>
-      <c r="K7" s="31"/>
-      <c r="L7" s="31"/>
-      <c r="M7" s="31"/>
-      <c r="N7" s="31"/>
-      <c r="O7" s="31"/>
-      <c r="P7" s="31"/>
-      <c r="Q7" s="31"/>
-      <c r="R7" s="31"/>
-      <c r="S7" s="31"/>
-      <c r="T7" s="31"/>
-      <c r="U7" s="31"/>
-      <c r="V7" s="31"/>
-      <c r="W7" s="31"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="28"/>
+      <c r="M7" s="28"/>
+      <c r="N7" s="28"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
+      <c r="R7" s="28"/>
+      <c r="S7" s="28"/>
+      <c r="T7" s="28"/>
+      <c r="U7" s="28"/>
+      <c r="V7" s="28"/>
+      <c r="W7" s="28"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="35" t="s">
+      <c r="A8" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="36"/>
-      <c r="J8" s="36"/>
-      <c r="K8" s="36"/>
-      <c r="L8" s="36"/>
-      <c r="M8" s="36"/>
-      <c r="N8" s="36"/>
-      <c r="O8" s="36"/>
-      <c r="P8" s="36"/>
-      <c r="Q8" s="36"/>
-      <c r="R8" s="36"/>
-      <c r="S8" s="36"/>
-      <c r="T8" s="36"/>
-      <c r="U8" s="36"/>
-      <c r="V8" s="36"/>
-      <c r="W8" s="36"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="33"/>
+      <c r="K8" s="33"/>
+      <c r="L8" s="33"/>
+      <c r="M8" s="33"/>
+      <c r="N8" s="33"/>
+      <c r="O8" s="33"/>
+      <c r="P8" s="33"/>
+      <c r="Q8" s="33"/>
+      <c r="R8" s="33"/>
+      <c r="S8" s="33"/>
+      <c r="T8" s="33"/>
+      <c r="U8" s="33"/>
+      <c r="V8" s="33"/>
+      <c r="W8" s="33"/>
     </row>
     <row r="9" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="35"/>
-      <c r="B9" s="31"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="31"/>
-      <c r="L9" s="31"/>
-      <c r="M9" s="31"/>
-      <c r="N9" s="31"/>
-      <c r="O9" s="31"/>
-      <c r="P9" s="31"/>
-      <c r="Q9" s="31"/>
-      <c r="R9" s="31"/>
-      <c r="S9" s="31"/>
-      <c r="T9" s="31"/>
-      <c r="U9" s="31"/>
-      <c r="V9" s="31"/>
-      <c r="W9" s="31"/>
+      <c r="A9" s="32"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="28"/>
+      <c r="K9" s="28"/>
+      <c r="L9" s="28"/>
+      <c r="M9" s="28"/>
+      <c r="N9" s="28"/>
+      <c r="O9" s="28"/>
+      <c r="P9" s="28"/>
+      <c r="Q9" s="28"/>
+      <c r="R9" s="28"/>
+      <c r="S9" s="28"/>
+      <c r="T9" s="28"/>
+      <c r="U9" s="28"/>
+      <c r="V9" s="28"/>
+      <c r="W9" s="28"/>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A10" s="31"/>
-      <c r="B10" s="31"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="31"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="31"/>
-      <c r="J10" s="31"/>
-      <c r="K10" s="31"/>
-      <c r="L10" s="31"/>
-      <c r="M10" s="31"/>
-      <c r="N10" s="31"/>
-      <c r="O10" s="31"/>
-      <c r="P10" s="31"/>
-      <c r="Q10" s="31"/>
-      <c r="R10" s="31"/>
-      <c r="S10" s="31"/>
-      <c r="T10" s="31"/>
-      <c r="U10" s="31"/>
-      <c r="V10" s="31"/>
-      <c r="W10" s="31"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="28"/>
+      <c r="L10" s="28"/>
+      <c r="M10" s="28"/>
+      <c r="N10" s="28"/>
+      <c r="O10" s="28"/>
+      <c r="P10" s="28"/>
+      <c r="Q10" s="28"/>
+      <c r="R10" s="28"/>
+      <c r="S10" s="28"/>
+      <c r="T10" s="28"/>
+      <c r="U10" s="28"/>
+      <c r="V10" s="28"/>
+      <c r="W10" s="28"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="31"/>
-      <c r="B11" s="31"/>
-      <c r="C11" s="38">
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="35">
         <v>2000</v>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="35">
         <v>2001</v>
       </c>
-      <c r="E11" s="38">
+      <c r="E11" s="35">
         <v>2002</v>
       </c>
-      <c r="F11" s="38">
+      <c r="F11" s="35">
         <v>2003</v>
       </c>
-      <c r="G11" s="38">
+      <c r="G11" s="35">
         <v>2004</v>
       </c>
-      <c r="H11" s="38">
+      <c r="H11" s="35">
         <v>2005</v>
       </c>
-      <c r="I11" s="38">
+      <c r="I11" s="35">
         <v>2006</v>
       </c>
-      <c r="J11" s="38">
+      <c r="J11" s="35">
         <v>2007</v>
       </c>
-      <c r="K11" s="38">
+      <c r="K11" s="35">
         <v>2008</v>
       </c>
-      <c r="L11" s="38">
+      <c r="L11" s="35">
         <v>2009</v>
       </c>
-      <c r="M11" s="38">
+      <c r="M11" s="35">
         <v>2010</v>
       </c>
-      <c r="N11" s="38">
+      <c r="N11" s="35">
         <v>2011</v>
       </c>
-      <c r="O11" s="38">
+      <c r="O11" s="35">
         <v>2012</v>
       </c>
-      <c r="P11" s="38">
+      <c r="P11" s="35">
         <v>2013</v>
       </c>
-      <c r="Q11" s="38">
+      <c r="Q11" s="35">
         <v>2014</v>
       </c>
-      <c r="R11" s="38">
+      <c r="R11" s="35">
         <v>2015</v>
       </c>
-      <c r="S11" s="38">
+      <c r="S11" s="35">
         <v>2016</v>
       </c>
-      <c r="T11" s="38">
+      <c r="T11" s="35">
         <v>2017</v>
       </c>
-      <c r="U11" s="38">
+      <c r="U11" s="35">
         <v>2018</v>
       </c>
-      <c r="V11" s="38">
+      <c r="V11" s="35">
         <v>2019</v>
       </c>
-      <c r="W11" s="38">
+      <c r="W11" s="35">
         <v>2020</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A12" s="31"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39"/>
-      <c r="J12" s="39"/>
-      <c r="K12" s="39"/>
-      <c r="L12" s="39"/>
-      <c r="M12" s="39"/>
-      <c r="N12" s="39"/>
-      <c r="O12" s="39"/>
-      <c r="P12" s="39"/>
-      <c r="Q12" s="39"/>
-      <c r="R12" s="39"/>
-      <c r="S12" s="39"/>
-      <c r="T12" s="31"/>
-      <c r="U12" s="31"/>
-      <c r="V12" s="31"/>
-      <c r="W12" s="31"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="36"/>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="36"/>
+      <c r="L12" s="36"/>
+      <c r="M12" s="36"/>
+      <c r="N12" s="36"/>
+      <c r="O12" s="36"/>
+      <c r="P12" s="36"/>
+      <c r="Q12" s="36"/>
+      <c r="R12" s="36"/>
+      <c r="S12" s="36"/>
+      <c r="T12" s="28"/>
+      <c r="U12" s="28"/>
+      <c r="V12" s="28"/>
+      <c r="W12" s="28"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A13" s="39"/>
-      <c r="B13" s="40" t="s">
+      <c r="A13" s="36"/>
+      <c r="B13" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="41">
+      <c r="C13" s="38">
         <v>2689</v>
       </c>
-      <c r="D13" s="41">
+      <c r="D13" s="38">
         <v>2783</v>
       </c>
-      <c r="E13" s="41">
+      <c r="E13" s="38">
         <v>2905</v>
       </c>
-      <c r="F13" s="41">
+      <c r="F13" s="38">
         <v>3006</v>
       </c>
-      <c r="G13" s="41">
+      <c r="G13" s="38">
         <v>3187</v>
       </c>
-      <c r="H13" s="41">
+      <c r="H13" s="38">
         <v>3338</v>
       </c>
-      <c r="I13" s="41">
+      <c r="I13" s="38">
         <v>3599.9839999999999</v>
       </c>
-      <c r="J13" s="41">
+      <c r="J13" s="38">
         <v>3606.5050000000001</v>
       </c>
-      <c r="K13" s="41">
+      <c r="K13" s="38">
         <v>3762</v>
       </c>
-      <c r="L13" s="41">
+      <c r="L13" s="38">
         <v>3767.46</v>
       </c>
-      <c r="M13" s="41">
+      <c r="M13" s="38">
         <v>3848.4679999999998</v>
       </c>
-      <c r="N13" s="41">
+      <c r="N13" s="38">
         <v>3928.9450000000002</v>
       </c>
-      <c r="O13" s="41">
+      <c r="O13" s="38">
         <v>3972.1790000000001</v>
       </c>
-      <c r="P13" s="41">
+      <c r="P13" s="38">
         <v>4052.9229999999998</v>
       </c>
-      <c r="Q13" s="41">
+      <c r="Q13" s="38">
         <v>4114.7790000000005</v>
       </c>
-      <c r="R13" s="41">
+      <c r="R13" s="38">
         <v>4176.7669999999998</v>
       </c>
-      <c r="S13" s="41">
+      <c r="S13" s="38">
         <v>4248.067</v>
       </c>
-      <c r="T13" s="41">
+      <c r="T13" s="38">
         <v>4309.9889999999996</v>
       </c>
-      <c r="U13" s="41">
+      <c r="U13" s="38">
         <v>4376.6329999999998</v>
       </c>
-      <c r="V13" s="41">
+      <c r="V13" s="38">
         <v>4443.2430000000004</v>
       </c>
-      <c r="W13" s="41">
+      <c r="W13" s="38">
         <v>4507.5259999999998</v>
       </c>
     </row>
     <row r="14" spans="1:23" ht="77.25" x14ac:dyDescent="0.25">
-      <c r="A14" s="31"/>
-      <c r="B14" s="42" t="s">
+      <c r="A14" s="28"/>
+      <c r="B14" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="43"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="43"/>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43"/>
-      <c r="K14" s="43"/>
-      <c r="L14" s="43"/>
-      <c r="M14" s="43"/>
-      <c r="N14" s="43"/>
-      <c r="O14" s="43"/>
-      <c r="P14" s="43"/>
-      <c r="Q14" s="43"/>
-      <c r="R14" s="43"/>
-      <c r="S14" s="43"/>
-      <c r="T14" s="43"/>
-      <c r="U14" s="43"/>
-      <c r="V14" s="43"/>
-      <c r="W14" s="43"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="40"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="40"/>
+      <c r="J14" s="40"/>
+      <c r="K14" s="40"/>
+      <c r="L14" s="40"/>
+      <c r="M14" s="40"/>
+      <c r="N14" s="40"/>
+      <c r="O14" s="40"/>
+      <c r="P14" s="40"/>
+      <c r="Q14" s="40"/>
+      <c r="R14" s="40"/>
+      <c r="S14" s="40"/>
+      <c r="T14" s="40"/>
+      <c r="U14" s="40"/>
+      <c r="V14" s="40"/>
+      <c r="W14" s="40"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A15" s="31"/>
-      <c r="B15" s="44" t="s">
+      <c r="A15" s="28"/>
+      <c r="B15" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="43">
+      <c r="C15" s="40">
         <v>751</v>
       </c>
-      <c r="D15" s="43">
+      <c r="D15" s="40">
         <v>776</v>
       </c>
-      <c r="E15" s="43">
+      <c r="E15" s="40">
         <v>845</v>
       </c>
-      <c r="F15" s="43">
+      <c r="F15" s="40">
         <v>796</v>
       </c>
-      <c r="G15" s="43">
+      <c r="G15" s="40">
         <v>790</v>
       </c>
-      <c r="H15" s="43">
+      <c r="H15" s="40">
         <v>827</v>
       </c>
-      <c r="I15" s="43">
+      <c r="I15" s="40">
         <v>985.25900000000001</v>
       </c>
-      <c r="J15" s="43">
+      <c r="J15" s="40">
         <v>965.25599999999997</v>
       </c>
-      <c r="K15" s="43">
+      <c r="K15" s="40">
         <v>944</v>
       </c>
-      <c r="L15" s="43">
+      <c r="L15" s="40">
         <v>881.21900000000005</v>
       </c>
-      <c r="M15" s="43">
+      <c r="M15" s="40">
         <v>860.59</v>
       </c>
-      <c r="N15" s="43">
+      <c r="N15" s="40">
         <v>818.57100000000003</v>
       </c>
-      <c r="O15" s="43">
+      <c r="O15" s="40">
         <v>776.86599999999999</v>
       </c>
-      <c r="P15" s="43">
+      <c r="P15" s="40">
         <v>745.54300000000001</v>
       </c>
-      <c r="Q15" s="43">
+      <c r="Q15" s="40">
         <v>703.68100000000004</v>
       </c>
-      <c r="R15" s="43">
+      <c r="R15" s="40">
         <v>667.16600000000005</v>
       </c>
-      <c r="S15" s="43">
+      <c r="S15" s="40">
         <v>630.57399999999996</v>
       </c>
-      <c r="T15" s="43">
+      <c r="T15" s="40">
         <v>591.38499999999999</v>
       </c>
-      <c r="U15" s="43">
+      <c r="U15" s="40">
         <v>554.83199999999999</v>
       </c>
-      <c r="V15" s="43">
+      <c r="V15" s="40">
         <v>516.94100000000003</v>
       </c>
-      <c r="W15" s="43">
+      <c r="W15" s="40">
         <v>479.07</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A16" s="31"/>
-      <c r="B16" s="44" t="s">
+      <c r="A16" s="28"/>
+      <c r="B16" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="43">
+      <c r="C16" s="40">
         <v>1938</v>
       </c>
-      <c r="D16" s="43">
+      <c r="D16" s="40">
         <v>2007</v>
       </c>
-      <c r="E16" s="43">
+      <c r="E16" s="40">
         <v>2060</v>
       </c>
-      <c r="F16" s="43">
+      <c r="F16" s="40">
         <v>2210</v>
       </c>
-      <c r="G16" s="43">
+      <c r="G16" s="40">
         <v>2397</v>
       </c>
-      <c r="H16" s="43">
+      <c r="H16" s="40">
         <v>2511</v>
       </c>
-      <c r="I16" s="43">
+      <c r="I16" s="40">
         <v>2614.7249999999999</v>
       </c>
-      <c r="J16" s="43">
+      <c r="J16" s="40">
         <v>2641.2489999999998</v>
       </c>
-      <c r="K16" s="43">
+      <c r="K16" s="40">
         <v>2818</v>
       </c>
-      <c r="L16" s="43">
+      <c r="L16" s="40">
         <v>2886.241</v>
       </c>
-      <c r="M16" s="43">
+      <c r="M16" s="40">
         <v>2987.8780000000002</v>
       </c>
-      <c r="N16" s="43">
+      <c r="N16" s="40">
         <v>3110.3739999999998</v>
       </c>
-      <c r="O16" s="43">
+      <c r="O16" s="40">
         <v>3195.3130000000001</v>
       </c>
-      <c r="P16" s="43">
+      <c r="P16" s="40">
         <v>3307.38</v>
       </c>
-      <c r="Q16" s="43">
+      <c r="Q16" s="40">
         <v>3411.098</v>
       </c>
-      <c r="R16" s="43">
+      <c r="R16" s="40">
         <v>3509.6010000000001</v>
       </c>
-      <c r="S16" s="43">
+      <c r="S16" s="40">
         <v>3617.4929999999999</v>
       </c>
-      <c r="T16" s="43">
+      <c r="T16" s="40">
         <v>3718.6039999999998</v>
       </c>
-      <c r="U16" s="43">
+      <c r="U16" s="40">
         <v>3821.8009999999999</v>
       </c>
-      <c r="V16" s="43">
+      <c r="V16" s="40">
         <v>3926.3020000000001</v>
       </c>
-      <c r="W16" s="43">
+      <c r="W16" s="40">
         <v>4028.4560000000001</v>
       </c>
     </row>
     <row r="17" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B17" s="31"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="43"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="43"/>
-      <c r="I17" s="43"/>
-      <c r="J17" s="43"/>
-      <c r="K17" s="43"/>
-      <c r="L17" s="43"/>
-      <c r="M17" s="43"/>
-      <c r="N17" s="43"/>
-      <c r="O17" s="43"/>
-      <c r="P17" s="43"/>
-      <c r="Q17" s="43"/>
-      <c r="R17" s="43"/>
-      <c r="S17" s="43"/>
-      <c r="T17" s="43"/>
-      <c r="U17" s="43"/>
-      <c r="V17" s="43"/>
-      <c r="W17" s="43"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="40"/>
+      <c r="I17" s="40"/>
+      <c r="J17" s="40"/>
+      <c r="K17" s="40"/>
+      <c r="L17" s="40"/>
+      <c r="M17" s="40"/>
+      <c r="N17" s="40"/>
+      <c r="O17" s="40"/>
+      <c r="P17" s="40"/>
+      <c r="Q17" s="40"/>
+      <c r="R17" s="40"/>
+      <c r="S17" s="40"/>
+      <c r="T17" s="40"/>
+      <c r="U17" s="40"/>
+      <c r="V17" s="40"/>
+      <c r="W17" s="40"/>
     </row>
     <row r="18" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B18" s="45" t="s">
+      <c r="B18" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="43"/>
-      <c r="I18" s="43"/>
-      <c r="J18" s="43"/>
-      <c r="K18" s="43"/>
-      <c r="L18" s="43"/>
-      <c r="M18" s="43"/>
-      <c r="N18" s="43"/>
-      <c r="O18" s="43"/>
-      <c r="P18" s="43"/>
-      <c r="Q18" s="43"/>
-      <c r="R18" s="43"/>
-      <c r="S18" s="43"/>
-      <c r="T18" s="43"/>
-      <c r="U18" s="43"/>
-      <c r="V18" s="43"/>
-      <c r="W18" s="43"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="40"/>
+      <c r="K18" s="40"/>
+      <c r="L18" s="40"/>
+      <c r="M18" s="40"/>
+      <c r="N18" s="40"/>
+      <c r="O18" s="40"/>
+      <c r="P18" s="40"/>
+      <c r="Q18" s="40"/>
+      <c r="R18" s="40"/>
+      <c r="S18" s="40"/>
+      <c r="T18" s="40"/>
+      <c r="U18" s="40"/>
+      <c r="V18" s="40"/>
+      <c r="W18" s="40"/>
     </row>
     <row r="19" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B19" s="44" t="s">
+      <c r="B19" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="43">
+      <c r="C19" s="40">
         <v>27.928598000000001</v>
       </c>
-      <c r="D19" s="43">
+      <c r="D19" s="40">
         <v>27.883579000000001</v>
       </c>
-      <c r="E19" s="43">
+      <c r="E19" s="40">
         <v>29.087779999999999</v>
       </c>
-      <c r="F19" s="43">
+      <c r="F19" s="40">
         <v>26.480373</v>
       </c>
-      <c r="G19" s="43">
+      <c r="G19" s="40">
         <v>24.788201999999998</v>
       </c>
-      <c r="H19" s="43">
+      <c r="H19" s="40">
         <v>24.775314999999999</v>
       </c>
-      <c r="I19" s="43">
+      <c r="I19" s="40">
         <v>27.368427000000001</v>
       </c>
-      <c r="J19" s="43">
+      <c r="J19" s="40">
         <v>26.764305</v>
       </c>
-      <c r="K19" s="43">
+      <c r="K19" s="40">
         <v>25.093036000000001</v>
       </c>
-      <c r="L19" s="43">
+      <c r="L19" s="40">
         <v>23.390267999999999</v>
       </c>
-      <c r="M19" s="43">
+      <c r="M19" s="40">
         <v>22.361885000000001</v>
       </c>
-      <c r="N19" s="43">
+      <c r="N19" s="40">
         <v>20.834371999999998</v>
       </c>
-      <c r="O19" s="43">
+      <c r="O19" s="40">
         <v>19.557679</v>
       </c>
-      <c r="P19" s="43">
+      <c r="P19" s="40">
         <v>18.395192999999999</v>
       </c>
-      <c r="Q19" s="43">
+      <c r="Q19" s="40">
         <v>17.101306999999998</v>
       </c>
-      <c r="R19" s="43">
+      <c r="R19" s="40">
         <v>15.973264</v>
       </c>
-      <c r="S19" s="43">
+      <c r="S19" s="40">
         <v>14.843787000000001</v>
       </c>
-      <c r="T19" s="43">
+      <c r="T19" s="40">
         <v>13.721265000000001</v>
       </c>
-      <c r="U19" s="43">
+      <c r="U19" s="40">
         <v>12.677142</v>
       </c>
-      <c r="V19" s="43">
+      <c r="V19" s="40">
         <v>11.634318</v>
       </c>
-      <c r="W19" s="43">
+      <c r="W19" s="40">
         <v>10.628225</v>
       </c>
     </row>
     <row r="20" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B20" s="44" t="s">
+      <c r="B20" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="43">
+      <c r="C20" s="40">
         <v>72.071402000000006</v>
       </c>
-      <c r="D20" s="43">
+      <c r="D20" s="40">
         <v>72.116421000000003</v>
       </c>
-      <c r="E20" s="43">
+      <c r="E20" s="40">
         <v>70.912220000000005</v>
       </c>
-      <c r="F20" s="43">
+      <c r="F20" s="40">
         <v>73.519627</v>
       </c>
-      <c r="G20" s="43">
+      <c r="G20" s="40">
         <v>75.211798000000002</v>
       </c>
-      <c r="H20" s="43">
+      <c r="H20" s="40">
         <v>75.224684999999994</v>
       </c>
-      <c r="I20" s="43">
+      <c r="I20" s="40">
         <v>72.631573000000003</v>
       </c>
-      <c r="J20" s="43">
+      <c r="J20" s="40">
         <v>73.235695000000007</v>
       </c>
-      <c r="K20" s="43">
+      <c r="K20" s="40">
         <v>74.906964000000002</v>
       </c>
-      <c r="L20" s="43">
+      <c r="L20" s="40">
         <v>76.609731999999994</v>
       </c>
-      <c r="M20" s="43">
+      <c r="M20" s="40">
         <v>77.638114999999999</v>
       </c>
-      <c r="N20" s="43">
+      <c r="N20" s="40">
         <v>79.165627999999998</v>
       </c>
-      <c r="O20" s="43">
+      <c r="O20" s="40">
         <v>80.442321000000007</v>
       </c>
-      <c r="P20" s="43">
+      <c r="P20" s="40">
         <v>81.604806999999994</v>
       </c>
-      <c r="Q20" s="43">
+      <c r="Q20" s="40">
         <v>82.898692999999994</v>
       </c>
-      <c r="R20" s="43">
+      <c r="R20" s="40">
         <v>84.026736</v>
       </c>
-      <c r="S20" s="43">
+      <c r="S20" s="40">
         <v>85.156212999999994</v>
       </c>
-      <c r="T20" s="43">
+      <c r="T20" s="40">
         <v>86.278734999999998</v>
       </c>
-      <c r="U20" s="43">
+      <c r="U20" s="40">
         <v>87.322857999999997</v>
       </c>
-      <c r="V20" s="43">
+      <c r="V20" s="40">
         <v>88.365682000000007</v>
       </c>
-      <c r="W20" s="43">
+      <c r="W20" s="40">
         <v>89.371775</v>
       </c>
     </row>
     <row r="21" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B21" s="31"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="43"/>
-      <c r="I21" s="43"/>
-      <c r="J21" s="43"/>
-      <c r="K21" s="43"/>
-      <c r="L21" s="43"/>
-      <c r="M21" s="43"/>
-      <c r="N21" s="43"/>
-      <c r="O21" s="43"/>
-      <c r="P21" s="43"/>
-      <c r="Q21" s="43"/>
-      <c r="R21" s="43"/>
-      <c r="S21" s="43"/>
-      <c r="T21" s="43"/>
-      <c r="U21" s="43"/>
-      <c r="V21" s="43"/>
-      <c r="W21" s="43"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="40"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40"/>
+      <c r="J21" s="40"/>
+      <c r="K21" s="40"/>
+      <c r="L21" s="40"/>
+      <c r="M21" s="40"/>
+      <c r="N21" s="40"/>
+      <c r="O21" s="40"/>
+      <c r="P21" s="40"/>
+      <c r="Q21" s="40"/>
+      <c r="R21" s="40"/>
+      <c r="S21" s="40"/>
+      <c r="T21" s="40"/>
+      <c r="U21" s="40"/>
+      <c r="V21" s="40"/>
+      <c r="W21" s="40"/>
     </row>
     <row r="22" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B22" s="46" t="s">
+      <c r="B22" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="43"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="43"/>
-      <c r="H22" s="43"/>
-      <c r="I22" s="43"/>
-      <c r="J22" s="43"/>
-      <c r="K22" s="43"/>
-      <c r="L22" s="43"/>
-      <c r="M22" s="43"/>
-      <c r="N22" s="43"/>
-      <c r="O22" s="43"/>
-      <c r="P22" s="43"/>
-      <c r="Q22" s="43"/>
-      <c r="R22" s="43"/>
-      <c r="S22" s="43"/>
-      <c r="T22" s="43"/>
-      <c r="U22" s="43"/>
-      <c r="V22" s="43"/>
-      <c r="W22" s="43"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="40"/>
+      <c r="J22" s="40"/>
+      <c r="K22" s="40"/>
+      <c r="L22" s="40"/>
+      <c r="M22" s="40"/>
+      <c r="N22" s="40"/>
+      <c r="O22" s="40"/>
+      <c r="P22" s="40"/>
+      <c r="Q22" s="40"/>
+      <c r="R22" s="40"/>
+      <c r="S22" s="40"/>
+      <c r="T22" s="40"/>
+      <c r="U22" s="40"/>
+      <c r="V22" s="40"/>
+      <c r="W22" s="40"/>
     </row>
     <row r="23" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B23" s="44" t="s">
+      <c r="B23" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="C23" s="43">
+      <c r="C23" s="40">
         <v>9.35</v>
       </c>
-      <c r="D23" s="43">
+      <c r="D23" s="40">
         <v>9.35</v>
       </c>
-      <c r="E23" s="43">
+      <c r="E23" s="40">
         <v>9.35</v>
       </c>
-      <c r="F23" s="43">
+      <c r="F23" s="40">
         <v>9.35</v>
       </c>
-      <c r="G23" s="43">
+      <c r="G23" s="40">
         <v>9.35</v>
       </c>
-      <c r="H23" s="43">
+      <c r="H23" s="40">
         <v>9.35</v>
       </c>
-      <c r="I23" s="43">
+      <c r="I23" s="40">
         <v>10.9</v>
       </c>
-      <c r="J23" s="43">
+      <c r="J23" s="40">
         <v>10.9</v>
       </c>
-      <c r="K23" s="43">
+      <c r="K23" s="40">
         <v>10.9</v>
       </c>
-      <c r="L23" s="43">
+      <c r="L23" s="40">
         <v>10.9</v>
       </c>
-      <c r="M23" s="43">
+      <c r="M23" s="40">
         <v>12</v>
       </c>
-      <c r="N23" s="43">
+      <c r="N23" s="40">
         <v>12</v>
       </c>
-      <c r="O23" s="43">
+      <c r="O23" s="40">
         <v>12</v>
       </c>
-      <c r="P23" s="43">
+      <c r="P23" s="40">
         <v>12</v>
       </c>
-      <c r="Q23" s="43">
+      <c r="Q23" s="40">
         <v>12</v>
       </c>
-      <c r="R23" s="43">
+      <c r="R23" s="40">
         <v>12</v>
       </c>
-      <c r="S23" s="43">
+      <c r="S23" s="40">
         <v>12</v>
       </c>
-      <c r="T23" s="43">
+      <c r="T23" s="40">
         <v>12</v>
       </c>
-      <c r="U23" s="43">
+      <c r="U23" s="40">
         <v>12</v>
       </c>
-      <c r="V23" s="43">
+      <c r="V23" s="40">
         <v>12</v>
       </c>
-      <c r="W23" s="43">
+      <c r="W23" s="40">
         <v>12</v>
       </c>
     </row>
     <row r="24" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B24" s="44" t="s">
+      <c r="B24" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="43">
+      <c r="C24" s="40">
         <v>10.3</v>
       </c>
-      <c r="D24" s="43">
+      <c r="D24" s="40">
         <v>10.3</v>
       </c>
-      <c r="E24" s="43">
+      <c r="E24" s="40">
         <v>10.3</v>
       </c>
-      <c r="F24" s="43">
+      <c r="F24" s="40">
         <v>10.3</v>
       </c>
-      <c r="G24" s="43">
+      <c r="G24" s="40">
         <v>10.3</v>
       </c>
-      <c r="H24" s="43">
+      <c r="H24" s="40">
         <v>10.3</v>
       </c>
-      <c r="I24" s="43">
+      <c r="I24" s="40">
         <v>13</v>
       </c>
-      <c r="J24" s="43">
+      <c r="J24" s="40">
         <v>13</v>
       </c>
-      <c r="K24" s="43">
+      <c r="K24" s="40">
         <v>13</v>
       </c>
-      <c r="L24" s="43">
+      <c r="L24" s="40">
         <v>13</v>
       </c>
-      <c r="M24" s="43">
+      <c r="M24" s="40">
         <v>13</v>
       </c>
-      <c r="N24" s="43">
+      <c r="N24" s="40">
         <v>13</v>
       </c>
-      <c r="O24" s="43">
+      <c r="O24" s="40">
         <v>13</v>
       </c>
-      <c r="P24" s="43">
+      <c r="P24" s="40">
         <v>13</v>
       </c>
-      <c r="Q24" s="43">
+      <c r="Q24" s="40">
         <v>13</v>
       </c>
-      <c r="R24" s="43">
+      <c r="R24" s="40">
         <v>13</v>
       </c>
-      <c r="S24" s="43">
+      <c r="S24" s="40">
         <v>13</v>
       </c>
-      <c r="T24" s="43">
+      <c r="T24" s="40">
         <v>13</v>
       </c>
-      <c r="U24" s="43">
+      <c r="U24" s="40">
         <v>13</v>
       </c>
-      <c r="V24" s="43">
+      <c r="V24" s="40">
         <v>13</v>
       </c>
-      <c r="W24" s="43">
+      <c r="W24" s="40">
         <v>13</v>
       </c>
     </row>
     <row r="25" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B25" s="46"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="43"/>
-      <c r="I25" s="43"/>
-      <c r="J25" s="43"/>
-      <c r="K25" s="43"/>
-      <c r="L25" s="43"/>
-      <c r="M25" s="43"/>
-      <c r="N25" s="43"/>
-      <c r="O25" s="43"/>
-      <c r="P25" s="43"/>
-      <c r="Q25" s="43"/>
-      <c r="R25" s="43"/>
-      <c r="S25" s="43"/>
-      <c r="T25" s="43"/>
-      <c r="U25" s="43"/>
-      <c r="V25" s="43"/>
-      <c r="W25" s="43"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="40"/>
+      <c r="I25" s="40"/>
+      <c r="J25" s="40"/>
+      <c r="K25" s="40"/>
+      <c r="L25" s="40"/>
+      <c r="M25" s="40"/>
+      <c r="N25" s="40"/>
+      <c r="O25" s="40"/>
+      <c r="P25" s="40"/>
+      <c r="Q25" s="40"/>
+      <c r="R25" s="40"/>
+      <c r="S25" s="40"/>
+      <c r="T25" s="40"/>
+      <c r="U25" s="40"/>
+      <c r="V25" s="40"/>
+      <c r="W25" s="40"/>
     </row>
     <row r="26" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B26" s="47" t="s">
+      <c r="B26" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="C26" s="43"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="43"/>
-      <c r="I26" s="43"/>
-      <c r="J26" s="43"/>
-      <c r="K26" s="43"/>
-      <c r="L26" s="43"/>
-      <c r="M26" s="43"/>
-      <c r="N26" s="43"/>
-      <c r="O26" s="43"/>
-      <c r="P26" s="43"/>
-      <c r="Q26" s="43"/>
-      <c r="R26" s="43"/>
-      <c r="S26" s="43"/>
-      <c r="T26" s="43"/>
-      <c r="U26" s="43"/>
-      <c r="V26" s="43"/>
-      <c r="W26" s="43"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="40"/>
+      <c r="I26" s="40"/>
+      <c r="J26" s="40"/>
+      <c r="K26" s="40"/>
+      <c r="L26" s="40"/>
+      <c r="M26" s="40"/>
+      <c r="N26" s="40"/>
+      <c r="O26" s="40"/>
+      <c r="P26" s="40"/>
+      <c r="Q26" s="40"/>
+      <c r="R26" s="40"/>
+      <c r="S26" s="40"/>
+      <c r="T26" s="40"/>
+      <c r="U26" s="40"/>
+      <c r="V26" s="40"/>
+      <c r="W26" s="40"/>
     </row>
     <row r="27" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B27" s="44" t="s">
+      <c r="B27" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="C27" s="43">
+      <c r="C27" s="40">
         <v>8.254899</v>
       </c>
-      <c r="D27" s="43">
+      <c r="D27" s="40">
         <v>8.4073619999999991</v>
       </c>
-      <c r="E27" s="43">
+      <c r="E27" s="40">
         <v>8.5724540000000005</v>
       </c>
-      <c r="F27" s="43">
+      <c r="F27" s="40">
         <v>8.7537540000000007</v>
       </c>
-      <c r="G27" s="43">
+      <c r="G27" s="40">
         <v>8.9275710000000004</v>
       </c>
-      <c r="H27" s="43">
+      <c r="H27" s="40">
         <v>9.0872240000000009</v>
       </c>
-      <c r="I27" s="43">
+      <c r="I27" s="40">
         <v>9.4962630000000008</v>
       </c>
-      <c r="J27" s="43">
+      <c r="J27" s="40">
         <v>9.7930130000000002</v>
       </c>
-      <c r="K27" s="43">
+      <c r="K27" s="40">
         <v>9.9979700000000005</v>
       </c>
-      <c r="L27" s="43">
+      <c r="L27" s="40">
         <v>10.143787</v>
       </c>
-      <c r="M27" s="43">
+      <c r="M27" s="40">
         <v>10.411020000000001</v>
       </c>
-      <c r="N27" s="43">
+      <c r="N27" s="40">
         <v>10.646141999999999</v>
       </c>
-      <c r="O27" s="43">
+      <c r="O27" s="40">
         <v>10.847928</v>
       </c>
-      <c r="P27" s="43">
+      <c r="P27" s="40">
         <v>11.018858</v>
       </c>
-      <c r="Q27" s="43">
+      <c r="Q27" s="40">
         <v>11.163881</v>
       </c>
-      <c r="R27" s="43">
+      <c r="R27" s="40">
         <v>11.287236999999999</v>
       </c>
-      <c r="S27" s="43">
+      <c r="S27" s="40">
         <v>11.394584999999999</v>
       </c>
-      <c r="T27" s="43">
+      <c r="T27" s="40">
         <v>11.493143</v>
       </c>
-      <c r="U27" s="43">
+      <c r="U27" s="40">
         <v>11.586477</v>
       </c>
-      <c r="V27" s="43">
+      <c r="V27" s="40">
         <v>11.674761</v>
       </c>
-      <c r="W27" s="43">
+      <c r="W27" s="40">
         <v>11.755246</v>
       </c>
     </row>
     <row r="28" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B28" s="44" t="s">
+      <c r="B28" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="43">
+      <c r="C28" s="40">
         <v>9.5897089999999992</v>
       </c>
-      <c r="D28" s="43">
+      <c r="D28" s="40">
         <v>9.6586390000000009</v>
       </c>
-      <c r="E28" s="43">
+      <c r="E28" s="40">
         <v>9.7456560000000003</v>
       </c>
-      <c r="F28" s="43">
+      <c r="F28" s="40">
         <v>9.8394600000000008</v>
       </c>
-      <c r="G28" s="43">
+      <c r="G28" s="40">
         <v>9.9334860000000003</v>
       </c>
-      <c r="H28" s="43">
+      <c r="H28" s="40">
         <v>10.030915</v>
       </c>
-      <c r="I28" s="43">
+      <c r="I28" s="40">
         <v>10.273657999999999</v>
       </c>
-      <c r="J28" s="43">
+      <c r="J28" s="40">
         <v>10.497527</v>
       </c>
-      <c r="K28" s="43">
+      <c r="K28" s="40">
         <v>10.704959000000001</v>
       </c>
-      <c r="L28" s="43">
+      <c r="L28" s="40">
         <v>10.877649</v>
       </c>
-      <c r="M28" s="43">
+      <c r="M28" s="40">
         <v>11.055011</v>
       </c>
-      <c r="N28" s="43">
+      <c r="N28" s="40">
         <v>11.219061999999999</v>
       </c>
-      <c r="O28" s="43">
+      <c r="O28" s="40">
         <v>11.404553999999999</v>
       </c>
-      <c r="P28" s="43">
+      <c r="P28" s="40">
         <v>11.579781000000001</v>
       </c>
-      <c r="Q28" s="43">
+      <c r="Q28" s="40">
         <v>11.734743999999999</v>
       </c>
-      <c r="R28" s="43">
+      <c r="R28" s="40">
         <v>11.914078999999999</v>
       </c>
-      <c r="S28" s="43">
+      <c r="S28" s="40">
         <v>12.101099</v>
       </c>
-      <c r="T28" s="43">
+      <c r="T28" s="40">
         <v>12.287822999999999</v>
       </c>
-      <c r="U28" s="43">
+      <c r="U28" s="40">
         <v>12.483280000000001</v>
       </c>
-      <c r="V28" s="43">
+      <c r="V28" s="40">
         <v>12.667294999999999</v>
       </c>
-      <c r="W28" s="43">
+      <c r="W28" s="40">
         <v>12.824119</v>
       </c>
     </row>
     <row r="29" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B29" s="40"/>
-      <c r="C29" s="43"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="43"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="43"/>
-      <c r="H29" s="43"/>
-      <c r="I29" s="43"/>
-      <c r="J29" s="43"/>
-      <c r="K29" s="43"/>
-      <c r="L29" s="43"/>
-      <c r="M29" s="43"/>
-      <c r="N29" s="43"/>
-      <c r="O29" s="43"/>
-      <c r="P29" s="43"/>
-      <c r="Q29" s="43"/>
-      <c r="R29" s="43"/>
-      <c r="S29" s="43"/>
-      <c r="T29" s="43"/>
-      <c r="U29" s="43"/>
-      <c r="V29" s="43"/>
-      <c r="W29" s="43"/>
+      <c r="B29" s="37"/>
+      <c r="C29" s="40"/>
+      <c r="D29" s="40"/>
+      <c r="E29" s="40"/>
+      <c r="F29" s="40"/>
+      <c r="G29" s="40"/>
+      <c r="H29" s="40"/>
+      <c r="I29" s="40"/>
+      <c r="J29" s="40"/>
+      <c r="K29" s="40"/>
+      <c r="L29" s="40"/>
+      <c r="M29" s="40"/>
+      <c r="N29" s="40"/>
+      <c r="O29" s="40"/>
+      <c r="P29" s="40"/>
+      <c r="Q29" s="40"/>
+      <c r="R29" s="40"/>
+      <c r="S29" s="40"/>
+      <c r="T29" s="40"/>
+      <c r="U29" s="40"/>
+      <c r="V29" s="40"/>
+      <c r="W29" s="40"/>
     </row>
     <row r="30" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B30" s="39" t="s">
+      <c r="B30" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="C30" s="31"/>
-      <c r="D30" s="31"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="31"/>
-      <c r="H30" s="31"/>
-      <c r="I30" s="31"/>
-      <c r="J30" s="31"/>
-      <c r="K30" s="31"/>
-      <c r="L30" s="31"/>
-      <c r="M30" s="31"/>
-      <c r="N30" s="31"/>
-      <c r="O30" s="31"/>
-      <c r="P30" s="31"/>
-      <c r="Q30" s="31"/>
-      <c r="R30" s="31"/>
-      <c r="S30" s="31"/>
-      <c r="T30" s="31"/>
-      <c r="U30" s="31"/>
-      <c r="V30" s="31"/>
-      <c r="W30" s="31"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="28"/>
+      <c r="K30" s="28"/>
+      <c r="L30" s="28"/>
+      <c r="M30" s="28"/>
+      <c r="N30" s="28"/>
+      <c r="O30" s="28"/>
+      <c r="P30" s="28"/>
+      <c r="Q30" s="28"/>
+      <c r="R30" s="28"/>
+      <c r="S30" s="28"/>
+      <c r="T30" s="28"/>
+      <c r="U30" s="28"/>
+      <c r="V30" s="28"/>
+      <c r="W30" s="28"/>
     </row>
     <row r="31" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B31" s="44" t="s">
+      <c r="B31" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="C31" s="48">
+      <c r="C31" s="45">
         <v>9898</v>
       </c>
-      <c r="D31" s="48">
+      <c r="D31" s="45">
         <v>9829</v>
       </c>
-      <c r="E31" s="48">
+      <c r="E31" s="45">
         <v>9797</v>
       </c>
-      <c r="F31" s="48">
+      <c r="F31" s="45">
         <v>9717</v>
       </c>
-      <c r="G31" s="48">
+      <c r="G31" s="45">
         <v>9531</v>
       </c>
-      <c r="H31" s="48">
+      <c r="H31" s="45">
         <v>9345</v>
       </c>
-      <c r="I31" s="48">
+      <c r="I31" s="45">
         <v>9181</v>
       </c>
-      <c r="J31" s="48">
+      <c r="J31" s="45">
         <v>9015</v>
       </c>
-      <c r="K31" s="48">
+      <c r="K31" s="45">
         <v>9048</v>
       </c>
-      <c r="L31" s="48">
+      <c r="L31" s="45">
         <v>9064</v>
       </c>
-      <c r="M31" s="48">
+      <c r="M31" s="45">
         <v>9086</v>
       </c>
-      <c r="N31" s="48">
+      <c r="N31" s="45">
         <v>9080</v>
       </c>
-      <c r="O31" s="48">
+      <c r="O31" s="45">
         <v>9090</v>
       </c>
-      <c r="P31" s="48">
+      <c r="P31" s="45">
         <v>9101</v>
       </c>
-      <c r="Q31" s="48">
+      <c r="Q31" s="45">
         <v>9111</v>
       </c>
-      <c r="R31" s="48">
+      <c r="R31" s="45">
         <v>9121</v>
       </c>
-      <c r="S31" s="48">
+      <c r="S31" s="45">
         <v>9132</v>
       </c>
-      <c r="T31" s="48">
+      <c r="T31" s="45">
         <v>9142</v>
       </c>
-      <c r="U31" s="48">
+      <c r="U31" s="45">
         <v>9152</v>
       </c>
-      <c r="V31" s="48">
+      <c r="V31" s="45">
         <v>9162</v>
       </c>
-      <c r="W31" s="48">
+      <c r="W31" s="45">
         <v>9172</v>
       </c>
     </row>
     <row r="32" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B32" s="44" t="s">
+      <c r="B32" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="C32" s="48">
+      <c r="C32" s="45">
         <v>33466</v>
       </c>
-      <c r="D32" s="48">
+      <c r="D32" s="45">
         <v>33624</v>
       </c>
-      <c r="E32" s="48">
+      <c r="E32" s="45">
         <v>33768</v>
       </c>
-      <c r="F32" s="48">
+      <c r="F32" s="45">
         <v>33919</v>
       </c>
-      <c r="G32" s="48">
+      <c r="G32" s="45">
         <v>33389</v>
       </c>
-      <c r="H32" s="48">
+      <c r="H32" s="45">
         <v>32873</v>
       </c>
-      <c r="I32" s="48">
+      <c r="I32" s="45">
         <v>32372</v>
       </c>
-      <c r="J32" s="48">
+      <c r="J32" s="45">
         <v>31873</v>
       </c>
-      <c r="K32" s="48">
+      <c r="K32" s="45">
         <v>31872</v>
       </c>
-      <c r="L32" s="48">
+      <c r="L32" s="45">
         <v>31884</v>
       </c>
-      <c r="M32" s="48">
+      <c r="M32" s="45">
         <v>31886</v>
       </c>
-      <c r="N32" s="48">
+      <c r="N32" s="45">
         <v>33236</v>
       </c>
-      <c r="O32" s="48">
+      <c r="O32" s="45">
         <v>33225</v>
       </c>
-      <c r="P32" s="48">
+      <c r="P32" s="45">
         <v>33225</v>
       </c>
-      <c r="Q32" s="48">
+      <c r="Q32" s="45">
         <v>33220</v>
       </c>
-      <c r="R32" s="48">
+      <c r="R32" s="45">
         <v>33215</v>
       </c>
-      <c r="S32" s="48">
+      <c r="S32" s="45">
         <v>33213</v>
       </c>
-      <c r="T32" s="48">
+      <c r="T32" s="45">
         <v>33208</v>
       </c>
-      <c r="U32" s="48">
+      <c r="U32" s="45">
         <v>33205</v>
       </c>
-      <c r="V32" s="48">
+      <c r="V32" s="45">
         <v>33202</v>
       </c>
-      <c r="W32" s="48">
+      <c r="W32" s="45">
         <v>33199</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="31"/>
-      <c r="B33" s="40"/>
-      <c r="C33" s="49"/>
-      <c r="D33" s="49"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="49"/>
-      <c r="J33" s="49"/>
-      <c r="K33" s="49"/>
-      <c r="L33" s="49"/>
-      <c r="M33" s="49"/>
-      <c r="N33" s="49"/>
-      <c r="O33" s="49"/>
+      <c r="A33" s="28"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="46"/>
+      <c r="D33" s="46"/>
+      <c r="E33" s="46"/>
+      <c r="F33" s="46"/>
+      <c r="G33" s="46"/>
+      <c r="H33" s="46"/>
+      <c r="I33" s="46"/>
+      <c r="J33" s="46"/>
+      <c r="K33" s="46"/>
+      <c r="L33" s="46"/>
+      <c r="M33" s="46"/>
+      <c r="N33" s="46"/>
+      <c r="O33" s="46"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A34" s="31" t="s">
+      <c r="A34" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="31"/>
-      <c r="C34" s="31"/>
-      <c r="D34" s="31"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="31"/>
-      <c r="H34" s="31"/>
-      <c r="I34" s="31"/>
-      <c r="J34" s="31"/>
-      <c r="K34" s="31"/>
-      <c r="L34" s="31"/>
-      <c r="M34" s="31"/>
-      <c r="N34" s="31"/>
-      <c r="O34" s="31"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="28"/>
+      <c r="H34" s="28"/>
+      <c r="I34" s="28"/>
+      <c r="J34" s="28"/>
+      <c r="K34" s="28"/>
+      <c r="L34" s="28"/>
+      <c r="M34" s="28"/>
+      <c r="N34" s="28"/>
+      <c r="O34" s="28"/>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="31" t="s">
+      <c r="A35" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B35" s="31"/>
-      <c r="C35" s="31"/>
-      <c r="D35" s="31"/>
-      <c r="E35" s="31"/>
-      <c r="F35" s="31"/>
-      <c r="G35" s="31"/>
-      <c r="H35" s="31"/>
-      <c r="I35" s="31"/>
-      <c r="J35" s="31"/>
-      <c r="K35" s="31"/>
-      <c r="L35" s="31"/>
-      <c r="M35" s="31"/>
-      <c r="N35" s="31"/>
-      <c r="O35" s="31"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="28"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="28"/>
+      <c r="K35" s="28"/>
+      <c r="L35" s="28"/>
+      <c r="M35" s="28"/>
+      <c r="N35" s="28"/>
+      <c r="O35" s="28"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A36" s="31"/>
-      <c r="B36" s="31"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="31"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="31"/>
-      <c r="H36" s="31"/>
-      <c r="I36" s="31"/>
-      <c r="J36" s="31"/>
-      <c r="K36" s="31"/>
-      <c r="L36" s="31"/>
-      <c r="M36" s="31"/>
-      <c r="N36" s="31"/>
-      <c r="O36" s="31"/>
+      <c r="A36" s="28"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28"/>
+      <c r="G36" s="28"/>
+      <c r="H36" s="28"/>
+      <c r="I36" s="28"/>
+      <c r="J36" s="28"/>
+      <c r="K36" s="28"/>
+      <c r="L36" s="28"/>
+      <c r="M36" s="28"/>
+      <c r="N36" s="28"/>
+      <c r="O36" s="28"/>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" s="31"/>
-      <c r="B37" s="31"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="31"/>
-      <c r="E37" s="31"/>
-      <c r="F37" s="31"/>
-      <c r="G37" s="31"/>
-      <c r="H37" s="31"/>
-      <c r="I37" s="31"/>
-      <c r="J37" s="31"/>
-      <c r="K37" s="31"/>
-      <c r="L37" s="31"/>
-      <c r="M37" s="31"/>
-      <c r="N37" s="31"/>
-      <c r="O37" s="31"/>
+      <c r="A37" s="28"/>
+      <c r="B37" s="28"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="28"/>
+      <c r="G37" s="28"/>
+      <c r="H37" s="28"/>
+      <c r="I37" s="28"/>
+      <c r="J37" s="28"/>
+      <c r="K37" s="28"/>
+      <c r="L37" s="28"/>
+      <c r="M37" s="28"/>
+      <c r="N37" s="28"/>
+      <c r="O37" s="28"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A38" s="31"/>
-      <c r="B38" s="31"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="31"/>
-      <c r="E38" s="31"/>
-      <c r="F38" s="31"/>
-      <c r="G38" s="31"/>
-      <c r="H38" s="31"/>
-      <c r="I38" s="31"/>
-      <c r="J38" s="31"/>
-      <c r="K38" s="31"/>
-      <c r="L38" s="31"/>
-      <c r="M38" s="31"/>
-      <c r="N38" s="31"/>
-      <c r="O38" s="31"/>
+      <c r="A38" s="28"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="28"/>
+      <c r="G38" s="28"/>
+      <c r="H38" s="28"/>
+      <c r="I38" s="28"/>
+      <c r="J38" s="28"/>
+      <c r="K38" s="28"/>
+      <c r="L38" s="28"/>
+      <c r="M38" s="28"/>
+      <c r="N38" s="28"/>
+      <c r="O38" s="28"/>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A39" s="31"/>
-      <c r="B39" s="40"/>
-      <c r="C39" s="31"/>
-      <c r="D39" s="31"/>
-      <c r="E39" s="31"/>
-      <c r="F39" s="31"/>
-      <c r="G39" s="31"/>
-      <c r="H39" s="31"/>
-      <c r="I39" s="31"/>
-      <c r="J39" s="31"/>
-      <c r="K39" s="31"/>
-      <c r="L39" s="31"/>
-      <c r="M39" s="31"/>
-      <c r="N39" s="31"/>
-      <c r="O39" s="31"/>
+      <c r="A39" s="28"/>
+      <c r="B39" s="37"/>
+      <c r="C39" s="28"/>
+      <c r="D39" s="28"/>
+      <c r="E39" s="28"/>
+      <c r="F39" s="28"/>
+      <c r="G39" s="28"/>
+      <c r="H39" s="28"/>
+      <c r="I39" s="28"/>
+      <c r="J39" s="28"/>
+      <c r="K39" s="28"/>
+      <c r="L39" s="28"/>
+      <c r="M39" s="28"/>
+      <c r="N39" s="28"/>
+      <c r="O39" s="28"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A40" s="31"/>
-      <c r="B40" s="40"/>
-      <c r="C40" s="31"/>
-      <c r="D40" s="31"/>
-      <c r="E40" s="31"/>
-      <c r="F40" s="31"/>
-      <c r="G40" s="31"/>
-      <c r="H40" s="31"/>
-      <c r="I40" s="31"/>
-      <c r="J40" s="31"/>
-      <c r="K40" s="31"/>
-      <c r="L40" s="31"/>
-      <c r="M40" s="31"/>
-      <c r="N40" s="31"/>
-      <c r="O40" s="31"/>
+      <c r="A40" s="28"/>
+      <c r="B40" s="37"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="28"/>
+      <c r="I40" s="28"/>
+      <c r="J40" s="28"/>
+      <c r="K40" s="28"/>
+      <c r="L40" s="28"/>
+      <c r="M40" s="28"/>
+      <c r="N40" s="28"/>
+      <c r="O40" s="28"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41" s="31"/>
-      <c r="B41" s="31"/>
-      <c r="C41" s="31"/>
-      <c r="D41" s="31"/>
-      <c r="E41" s="31"/>
-      <c r="F41" s="31"/>
-      <c r="G41" s="31"/>
-      <c r="H41" s="31"/>
-      <c r="I41" s="31"/>
-      <c r="J41" s="31"/>
-      <c r="K41" s="31"/>
-      <c r="L41" s="31"/>
-      <c r="M41" s="31"/>
-      <c r="N41" s="31"/>
-      <c r="O41" s="31"/>
+      <c r="A41" s="28"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="28"/>
+      <c r="F41" s="28"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="28"/>
+      <c r="I41" s="28"/>
+      <c r="J41" s="28"/>
+      <c r="K41" s="28"/>
+      <c r="L41" s="28"/>
+      <c r="M41" s="28"/>
+      <c r="N41" s="28"/>
+      <c r="O41" s="28"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A42" s="31"/>
-      <c r="B42" s="31"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="31"/>
-      <c r="E42" s="31"/>
-      <c r="F42" s="31"/>
-      <c r="G42" s="31"/>
-      <c r="H42" s="31"/>
-      <c r="I42" s="31"/>
-      <c r="J42" s="31"/>
-      <c r="K42" s="31"/>
-      <c r="L42" s="31"/>
-      <c r="M42" s="31"/>
-      <c r="N42" s="31"/>
-      <c r="O42" s="31"/>
+      <c r="A42" s="28"/>
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="28"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="28"/>
+      <c r="I42" s="28"/>
+      <c r="J42" s="28"/>
+      <c r="K42" s="28"/>
+      <c r="L42" s="28"/>
+      <c r="M42" s="28"/>
+      <c r="N42" s="28"/>
+      <c r="O42" s="28"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="31"/>
-      <c r="B43" s="31"/>
-      <c r="C43" s="31"/>
-      <c r="D43" s="31"/>
-      <c r="E43" s="31"/>
-      <c r="F43" s="31"/>
-      <c r="G43" s="31"/>
-      <c r="H43" s="31"/>
-      <c r="I43" s="31"/>
-      <c r="J43" s="31"/>
-      <c r="K43" s="31"/>
-      <c r="L43" s="31"/>
-      <c r="M43" s="31"/>
-      <c r="N43" s="31"/>
-      <c r="O43" s="31"/>
+      <c r="A43" s="28"/>
+      <c r="B43" s="28"/>
+      <c r="C43" s="28"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="28"/>
+      <c r="F43" s="28"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="28"/>
+      <c r="I43" s="28"/>
+      <c r="J43" s="28"/>
+      <c r="K43" s="28"/>
+      <c r="L43" s="28"/>
+      <c r="M43" s="28"/>
+      <c r="N43" s="28"/>
+      <c r="O43" s="28"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A44" s="31"/>
-      <c r="B44" s="40"/>
-      <c r="C44" s="31"/>
-      <c r="D44" s="31"/>
-      <c r="E44" s="31"/>
-      <c r="F44" s="31"/>
-      <c r="G44" s="31"/>
-      <c r="H44" s="31"/>
-      <c r="I44" s="31"/>
-      <c r="J44" s="31"/>
-      <c r="K44" s="31"/>
-      <c r="L44" s="31"/>
-      <c r="M44" s="31"/>
-      <c r="N44" s="31"/>
-      <c r="O44" s="31"/>
+      <c r="A44" s="28"/>
+      <c r="B44" s="37"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="28"/>
+      <c r="F44" s="28"/>
+      <c r="G44" s="28"/>
+      <c r="H44" s="28"/>
+      <c r="I44" s="28"/>
+      <c r="J44" s="28"/>
+      <c r="K44" s="28"/>
+      <c r="L44" s="28"/>
+      <c r="M44" s="28"/>
+      <c r="N44" s="28"/>
+      <c r="O44" s="28"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A45" s="31"/>
-      <c r="B45" s="31"/>
-      <c r="C45" s="31"/>
-      <c r="D45" s="31"/>
-      <c r="E45" s="31"/>
-      <c r="F45" s="31"/>
-      <c r="G45" s="31"/>
-      <c r="H45" s="31"/>
-      <c r="I45" s="31"/>
-      <c r="J45" s="31"/>
-      <c r="K45" s="31"/>
-      <c r="L45" s="31"/>
-      <c r="M45" s="31"/>
-      <c r="N45" s="31"/>
-      <c r="O45" s="31"/>
+      <c r="A45" s="28"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="28"/>
+      <c r="G45" s="28"/>
+      <c r="H45" s="28"/>
+      <c r="I45" s="28"/>
+      <c r="J45" s="28"/>
+      <c r="K45" s="28"/>
+      <c r="L45" s="28"/>
+      <c r="M45" s="28"/>
+      <c r="N45" s="28"/>
+      <c r="O45" s="28"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A46" s="31"/>
-      <c r="B46" s="31"/>
-      <c r="C46" s="31"/>
-      <c r="D46" s="31"/>
-      <c r="E46" s="31"/>
-      <c r="F46" s="31"/>
-      <c r="G46" s="31"/>
-      <c r="H46" s="31"/>
-      <c r="I46" s="31"/>
-      <c r="J46" s="31"/>
-      <c r="K46" s="31"/>
-      <c r="L46" s="31"/>
-      <c r="M46" s="31"/>
-      <c r="N46" s="31"/>
-      <c r="O46" s="31"/>
+      <c r="A46" s="28"/>
+      <c r="B46" s="28"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="28"/>
+      <c r="E46" s="28"/>
+      <c r="F46" s="28"/>
+      <c r="G46" s="28"/>
+      <c r="H46" s="28"/>
+      <c r="I46" s="28"/>
+      <c r="J46" s="28"/>
+      <c r="K46" s="28"/>
+      <c r="L46" s="28"/>
+      <c r="M46" s="28"/>
+      <c r="N46" s="28"/>
+      <c r="O46" s="28"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A47" s="31"/>
-      <c r="B47" s="31"/>
-      <c r="C47" s="31"/>
-      <c r="D47" s="31"/>
-      <c r="E47" s="31"/>
-      <c r="F47" s="31"/>
-      <c r="G47" s="31"/>
-      <c r="H47" s="31"/>
-      <c r="I47" s="31"/>
-      <c r="J47" s="31"/>
-      <c r="K47" s="31"/>
-      <c r="L47" s="31"/>
-      <c r="M47" s="31"/>
-      <c r="N47" s="31"/>
-      <c r="O47" s="31"/>
+      <c r="A47" s="28"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="28"/>
+      <c r="E47" s="28"/>
+      <c r="F47" s="28"/>
+      <c r="G47" s="28"/>
+      <c r="H47" s="28"/>
+      <c r="I47" s="28"/>
+      <c r="J47" s="28"/>
+      <c r="K47" s="28"/>
+      <c r="L47" s="28"/>
+      <c r="M47" s="28"/>
+      <c r="N47" s="28"/>
+      <c r="O47" s="28"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" s="31"/>
-      <c r="B48" s="40"/>
-      <c r="C48" s="31"/>
-      <c r="D48" s="31"/>
-      <c r="E48" s="31"/>
-      <c r="F48" s="31"/>
-      <c r="G48" s="31"/>
-      <c r="H48" s="31"/>
-      <c r="I48" s="31"/>
-      <c r="J48" s="31"/>
-      <c r="K48" s="31"/>
-      <c r="L48" s="31"/>
-      <c r="M48" s="31"/>
-      <c r="N48" s="31"/>
-      <c r="O48" s="31"/>
+      <c r="A48" s="28"/>
+      <c r="B48" s="37"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="28"/>
+      <c r="E48" s="28"/>
+      <c r="F48" s="28"/>
+      <c r="G48" s="28"/>
+      <c r="H48" s="28"/>
+      <c r="I48" s="28"/>
+      <c r="J48" s="28"/>
+      <c r="K48" s="28"/>
+      <c r="L48" s="28"/>
+      <c r="M48" s="28"/>
+      <c r="N48" s="28"/>
+      <c r="O48" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>